<commit_message>
Deep refactoring of all modules following pylint code review
</commit_message>
<xml_diff>
--- a/BiblioParsing/BiblioParsing_RefFiles/Countries.xlsx
+++ b/BiblioParsing/BiblioParsing_RefFiles/Countries.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileSharing readOnlyRecommended="1"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AC265100\PyVenv\BiblioParsing\BiblioParsing\BiblioParsing_RefFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AC265100\Documents\BiblioMeter_App\LETI\Bibliometry\BiblioMeter_Files-6.2.0\Traitement Institutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C09BAFB1-03D3-4E61-BBA5-D2FCE3A0E395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C3F58D-C861-446F-90E8-A7371595AC71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27945" yWindow="8325" windowWidth="23775" windowHeight="12915" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34230" yWindow="10500" windowWidth="30480" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2648,17 +2649,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F231"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2678,7 +2679,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2698,7 +2699,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2718,7 +2719,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2738,7 +2739,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2758,7 +2759,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2798,7 +2799,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2818,7 +2819,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -2838,7 +2839,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -2858,7 +2859,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -2878,7 +2879,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2898,7 +2899,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -2918,7 +2919,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -2938,7 +2939,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -2958,7 +2959,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -2978,7 +2979,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -2998,7 +2999,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -3018,7 +3019,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -3038,7 +3039,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -3058,7 +3059,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -3078,7 +3079,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -3098,7 +3099,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -3118,7 +3119,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -3138,7 +3139,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -3158,7 +3159,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -3178,7 +3179,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -3198,7 +3199,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -3218,7 +3219,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -3238,7 +3239,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -3258,7 +3259,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -3278,7 +3279,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -3298,7 +3299,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -3318,7 +3319,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -3338,7 +3339,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -3358,7 +3359,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -3378,7 +3379,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -3398,7 +3399,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -3418,7 +3419,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -3438,7 +3439,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -3458,7 +3459,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -3478,7 +3479,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -3498,7 +3499,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -3518,7 +3519,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -3538,7 +3539,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -3558,7 +3559,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -3578,7 +3579,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -3598,7 +3599,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -3618,7 +3619,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -3638,7 +3639,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>736</v>
       </c>
@@ -3658,7 +3659,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -3678,7 +3679,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>55</v>
       </c>
@@ -3698,7 +3699,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -3718,7 +3719,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -3738,7 +3739,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -3758,7 +3759,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -3778,7 +3779,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -3798,7 +3799,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>61</v>
       </c>
@@ -3818,7 +3819,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>62</v>
       </c>
@@ -3838,7 +3839,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -3858,7 +3859,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>64</v>
       </c>
@@ -3878,7 +3879,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -3898,7 +3899,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>66</v>
       </c>
@@ -3918,7 +3919,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -3938,7 +3939,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -3958,7 +3959,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -3978,7 +3979,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>70</v>
       </c>
@@ -3998,7 +3999,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>71</v>
       </c>
@@ -4018,7 +4019,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>72</v>
       </c>
@@ -4038,7 +4039,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>73</v>
       </c>
@@ -4058,7 +4059,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>74</v>
       </c>
@@ -4078,7 +4079,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>75</v>
       </c>
@@ -4098,7 +4099,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>76</v>
       </c>
@@ -4118,7 +4119,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>77</v>
       </c>
@@ -4138,7 +4139,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>78</v>
       </c>
@@ -4158,7 +4159,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -4178,7 +4179,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>80</v>
       </c>
@@ -4198,7 +4199,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>81</v>
       </c>
@@ -4218,7 +4219,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>82</v>
       </c>
@@ -4238,7 +4239,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -4258,7 +4259,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -4278,7 +4279,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>85</v>
       </c>
@@ -4298,7 +4299,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>86</v>
       </c>
@@ -4318,7 +4319,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>87</v>
       </c>
@@ -4338,7 +4339,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>88</v>
       </c>
@@ -4358,7 +4359,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>89</v>
       </c>
@@ -4378,7 +4379,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>90</v>
       </c>
@@ -4398,7 +4399,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>91</v>
       </c>
@@ -4418,7 +4419,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>92</v>
       </c>
@@ -4438,7 +4439,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>93</v>
       </c>
@@ -4458,7 +4459,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>94</v>
       </c>
@@ -4478,7 +4479,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>95</v>
       </c>
@@ -4498,7 +4499,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -4518,7 +4519,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>97</v>
       </c>
@@ -4538,7 +4539,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>98</v>
       </c>
@@ -4558,7 +4559,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>99</v>
       </c>
@@ -4578,7 +4579,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>100</v>
       </c>
@@ -4598,7 +4599,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -4618,7 +4619,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -4638,7 +4639,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -4658,7 +4659,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -4678,7 +4679,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>105</v>
       </c>
@@ -4698,7 +4699,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>106</v>
       </c>
@@ -4718,7 +4719,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>107</v>
       </c>
@@ -4738,7 +4739,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>108</v>
       </c>
@@ -4758,7 +4759,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>109</v>
       </c>
@@ -4778,7 +4779,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>110</v>
       </c>
@@ -4798,7 +4799,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>111</v>
       </c>
@@ -4818,7 +4819,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>112</v>
       </c>
@@ -4838,7 +4839,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>113</v>
       </c>
@@ -4858,7 +4859,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>114</v>
       </c>
@@ -4878,7 +4879,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>115</v>
       </c>
@@ -4898,7 +4899,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>116</v>
       </c>
@@ -4918,7 +4919,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>117</v>
       </c>
@@ -4938,7 +4939,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>118</v>
       </c>
@@ -4958,7 +4959,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>119</v>
       </c>
@@ -4978,7 +4979,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>120</v>
       </c>
@@ -4998,7 +4999,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>121</v>
       </c>
@@ -5018,7 +5019,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>122</v>
       </c>
@@ -5038,7 +5039,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>123</v>
       </c>
@@ -5058,7 +5059,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>124</v>
       </c>
@@ -5078,7 +5079,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>125</v>
       </c>
@@ -5098,7 +5099,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>126</v>
       </c>
@@ -5118,7 +5119,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>127</v>
       </c>
@@ -5138,7 +5139,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>128</v>
       </c>
@@ -5158,7 +5159,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>129</v>
       </c>
@@ -5178,7 +5179,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>130</v>
       </c>
@@ -5198,7 +5199,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>131</v>
       </c>
@@ -5218,7 +5219,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>132</v>
       </c>
@@ -5238,7 +5239,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>133</v>
       </c>
@@ -5258,7 +5259,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>134</v>
       </c>
@@ -5278,7 +5279,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>135</v>
       </c>
@@ -5298,7 +5299,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>136</v>
       </c>
@@ -5318,7 +5319,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>137</v>
       </c>
@@ -5338,7 +5339,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>138</v>
       </c>
@@ -5358,7 +5359,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>139</v>
       </c>
@@ -5378,7 +5379,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>140</v>
       </c>
@@ -5398,7 +5399,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>141</v>
       </c>
@@ -5418,7 +5419,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>142</v>
       </c>
@@ -5438,7 +5439,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>143</v>
       </c>
@@ -5458,7 +5459,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>144</v>
       </c>
@@ -5478,7 +5479,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>145</v>
       </c>
@@ -5498,7 +5499,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>146</v>
       </c>
@@ -5518,7 +5519,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>147</v>
       </c>
@@ -5538,7 +5539,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>148</v>
       </c>
@@ -5558,7 +5559,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>149</v>
       </c>
@@ -5578,7 +5579,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>150</v>
       </c>
@@ -5598,7 +5599,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>151</v>
       </c>
@@ -5618,7 +5619,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>152</v>
       </c>
@@ -5638,7 +5639,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>153</v>
       </c>
@@ -5658,7 +5659,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>154</v>
       </c>
@@ -5678,7 +5679,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>155</v>
       </c>
@@ -5698,7 +5699,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>156</v>
       </c>
@@ -5718,7 +5719,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>157</v>
       </c>
@@ -5738,7 +5739,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>158</v>
       </c>
@@ -5758,7 +5759,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>159</v>
       </c>
@@ -5778,7 +5779,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>160</v>
       </c>
@@ -5798,7 +5799,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>161</v>
       </c>
@@ -5818,7 +5819,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>162</v>
       </c>
@@ -5838,7 +5839,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>163</v>
       </c>
@@ -5858,7 +5859,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>164</v>
       </c>
@@ -5878,7 +5879,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>165</v>
       </c>
@@ -5898,7 +5899,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>166</v>
       </c>
@@ -5918,7 +5919,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>167</v>
       </c>
@@ -5938,7 +5939,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>168</v>
       </c>
@@ -5958,7 +5959,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>169</v>
       </c>
@@ -5978,7 +5979,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>170</v>
       </c>
@@ -5998,7 +5999,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>171</v>
       </c>
@@ -6018,7 +6019,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>172</v>
       </c>
@@ -6038,7 +6039,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>173</v>
       </c>
@@ -6058,7 +6059,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>174</v>
       </c>
@@ -6078,7 +6079,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>175</v>
       </c>
@@ -6098,7 +6099,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>176</v>
       </c>
@@ -6118,7 +6119,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>177</v>
       </c>
@@ -6138,7 +6139,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>178</v>
       </c>
@@ -6158,7 +6159,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>179</v>
       </c>
@@ -6178,7 +6179,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>180</v>
       </c>
@@ -6198,7 +6199,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>181</v>
       </c>
@@ -6218,7 +6219,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>182</v>
       </c>
@@ -6238,7 +6239,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>183</v>
       </c>
@@ -6258,7 +6259,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>184</v>
       </c>
@@ -6278,7 +6279,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>185</v>
       </c>
@@ -6298,7 +6299,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>186</v>
       </c>
@@ -6318,7 +6319,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>187</v>
       </c>
@@ -6338,7 +6339,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>188</v>
       </c>
@@ -6358,7 +6359,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>189</v>
       </c>
@@ -6378,7 +6379,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>190</v>
       </c>
@@ -6398,7 +6399,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>191</v>
       </c>
@@ -6418,7 +6419,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>192</v>
       </c>
@@ -6438,7 +6439,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>193</v>
       </c>
@@ -6458,7 +6459,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>194</v>
       </c>
@@ -6478,7 +6479,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>195</v>
       </c>
@@ -6498,7 +6499,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>196</v>
       </c>
@@ -6518,7 +6519,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>197</v>
       </c>
@@ -6538,7 +6539,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>198</v>
       </c>
@@ -6558,7 +6559,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>199</v>
       </c>
@@ -6578,7 +6579,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>200</v>
       </c>
@@ -6598,7 +6599,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>201</v>
       </c>
@@ -6618,7 +6619,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>202</v>
       </c>
@@ -6638,7 +6639,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>203</v>
       </c>
@@ -6658,7 +6659,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>204</v>
       </c>
@@ -6678,7 +6679,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>205</v>
       </c>
@@ -6698,7 +6699,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>206</v>
       </c>
@@ -6718,7 +6719,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>207</v>
       </c>
@@ -6738,7 +6739,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>208</v>
       </c>
@@ -6758,7 +6759,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>209</v>
       </c>
@@ -6778,7 +6779,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>210</v>
       </c>
@@ -6798,7 +6799,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>211</v>
       </c>
@@ -6818,7 +6819,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>212</v>
       </c>
@@ -6838,7 +6839,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>213</v>
       </c>
@@ -6858,7 +6859,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>214</v>
       </c>
@@ -6878,7 +6879,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>215</v>
       </c>
@@ -6898,7 +6899,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>216</v>
       </c>
@@ -6918,7 +6919,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>217</v>
       </c>
@@ -6938,7 +6939,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>218</v>
       </c>
@@ -6958,7 +6959,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>219</v>
       </c>
@@ -6978,7 +6979,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>220</v>
       </c>
@@ -6998,7 +6999,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>221</v>
       </c>
@@ -7018,7 +7019,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>222</v>
       </c>
@@ -7038,7 +7039,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>223</v>
       </c>
@@ -7058,7 +7059,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>224</v>
       </c>
@@ -7078,7 +7079,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>225</v>
       </c>
@@ -7098,7 +7099,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
         <v>226</v>
       </c>
@@ -7118,7 +7119,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>227</v>
       </c>
@@ -7138,7 +7139,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>228</v>
       </c>
@@ -7158,7 +7159,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>229</v>
       </c>
@@ -7178,7 +7179,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>230</v>
       </c>
@@ -7198,7 +7199,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>231</v>
       </c>
@@ -7218,7 +7219,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>232</v>
       </c>
@@ -7238,7 +7239,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>233</v>
       </c>
@@ -7258,7 +7259,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>738</v>
       </c>

</xml_diff>